<commit_message>
fix: POR template bersih dari data lama + klasifikasi antibiotik pakai master Medisy + verifikasi simpan
</commit_message>
<xml_diff>
--- a/public/tpl_por.xlsx
+++ b/public/tpl_por.xlsx
@@ -1215,14 +1215,8 @@
       <c r="G10" s="42" t="n"/>
       <c r="H10" s="42" t="n"/>
       <c r="I10" s="34" t="n"/>
-      <c r="J10" s="42" t="inlineStr">
-        <is>
-          <t>3x1</t>
-        </is>
-      </c>
-      <c r="K10" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J10" s="42" t="n"/>
+      <c r="K10" s="42" t="n"/>
       <c r="L10" s="42" t="n"/>
       <c r="M10" s="42" t="n"/>
       <c r="N10" s="42" t="n"/>
@@ -1244,14 +1238,8 @@
       <c r="G11" s="68" t="n"/>
       <c r="H11" s="42" t="n"/>
       <c r="I11" s="34" t="n"/>
-      <c r="J11" s="42" t="inlineStr">
-        <is>
-          <t>1x1</t>
-        </is>
-      </c>
-      <c r="K11" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J11" s="42" t="n"/>
+      <c r="K11" s="42" t="n"/>
       <c r="L11" s="42" t="n"/>
       <c r="M11" s="42" t="n"/>
       <c r="T11" s="4" t="n"/>
@@ -1272,14 +1260,8 @@
       <c r="G12" s="68" t="n"/>
       <c r="H12" s="42" t="n"/>
       <c r="I12" s="34" t="n"/>
-      <c r="J12" s="42" t="inlineStr">
-        <is>
-          <t>3x1</t>
-        </is>
-      </c>
-      <c r="K12" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J12" s="42" t="n"/>
+      <c r="K12" s="42" t="n"/>
       <c r="L12" s="42" t="n"/>
       <c r="M12" s="42" t="n"/>
       <c r="T12" s="4" t="n"/>
@@ -1300,14 +1282,8 @@
       <c r="G13" s="69" t="n"/>
       <c r="H13" s="42" t="n"/>
       <c r="I13" s="34" t="n"/>
-      <c r="J13" s="42" t="inlineStr">
-        <is>
-          <t>3x1</t>
-        </is>
-      </c>
-      <c r="K13" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J13" s="42" t="n"/>
+      <c r="K13" s="42" t="n"/>
       <c r="L13" s="42" t="n"/>
       <c r="M13" s="42" t="n"/>
       <c r="T13" s="4" t="n"/>
@@ -1328,14 +1304,8 @@
       <c r="G14" s="42" t="n"/>
       <c r="H14" s="42" t="n"/>
       <c r="I14" s="42" t="n"/>
-      <c r="J14" s="42" t="inlineStr">
-        <is>
-          <t>1x1</t>
-        </is>
-      </c>
-      <c r="K14" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J14" s="42" t="n"/>
+      <c r="K14" s="42" t="n"/>
       <c r="L14" s="42" t="n"/>
       <c r="M14" s="42" t="n"/>
       <c r="N14" s="42" t="n"/>
@@ -1379,14 +1349,8 @@
       <c r="G16" s="69" t="n"/>
       <c r="H16" s="42" t="n"/>
       <c r="I16" s="42" t="n"/>
-      <c r="J16" s="42" t="inlineStr">
-        <is>
-          <t>2x1</t>
-        </is>
-      </c>
-      <c r="K16" s="42" t="n">
-        <v>1</v>
-      </c>
+      <c r="J16" s="42" t="n"/>
+      <c r="K16" s="42" t="n"/>
       <c r="L16" s="42" t="n"/>
       <c r="M16" s="42" t="n"/>
       <c r="T16" s="4" t="n"/>
@@ -1416,14 +1380,8 @@
       <c r="G18" s="42" t="n"/>
       <c r="H18" s="42" t="n"/>
       <c r="I18" s="42" t="n"/>
-      <c r="J18" s="42" t="inlineStr">
-        <is>
-          <t>1x1</t>
-        </is>
-      </c>
-      <c r="K18" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J18" s="42" t="n"/>
+      <c r="K18" s="42" t="n"/>
       <c r="L18" s="42" t="n"/>
       <c r="M18" s="42" t="n"/>
       <c r="N18" s="42" t="n"/>
@@ -1445,14 +1403,8 @@
       <c r="G19" s="68" t="n"/>
       <c r="H19" s="42" t="n"/>
       <c r="I19" s="42" t="n"/>
-      <c r="J19" s="42" t="inlineStr">
-        <is>
-          <t>2x1</t>
-        </is>
-      </c>
-      <c r="K19" s="42" t="n">
-        <v>1</v>
-      </c>
+      <c r="J19" s="42" t="n"/>
+      <c r="K19" s="42" t="n"/>
       <c r="L19" s="42" t="n"/>
       <c r="M19" s="42" t="n"/>
       <c r="T19" s="4" t="n"/>
@@ -1473,14 +1425,8 @@
       <c r="G20" s="68" t="n"/>
       <c r="H20" s="42" t="n"/>
       <c r="I20" s="42" t="n"/>
-      <c r="J20" s="42" t="inlineStr">
-        <is>
-          <t>3x1</t>
-        </is>
-      </c>
-      <c r="K20" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J20" s="42" t="n"/>
+      <c r="K20" s="42" t="n"/>
       <c r="L20" s="42" t="n"/>
       <c r="M20" s="42" t="n"/>
       <c r="T20" s="4" t="n"/>
@@ -1564,14 +1510,8 @@
       <c r="G25" s="68" t="n"/>
       <c r="H25" s="42" t="n"/>
       <c r="I25" s="42" t="n"/>
-      <c r="J25" s="42" t="inlineStr">
-        <is>
-          <t>1x1</t>
-        </is>
-      </c>
-      <c r="K25" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J25" s="42" t="n"/>
+      <c r="K25" s="42" t="n"/>
       <c r="L25" s="42" t="n"/>
       <c r="M25" s="42" t="n"/>
       <c r="T25" s="4" t="n"/>
@@ -1592,14 +1532,8 @@
       <c r="G26" s="68" t="n"/>
       <c r="H26" s="42" t="n"/>
       <c r="I26" s="42" t="n"/>
-      <c r="J26" s="42" t="inlineStr">
-        <is>
-          <t>3x1</t>
-        </is>
-      </c>
-      <c r="K26" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J26" s="42" t="n"/>
+      <c r="K26" s="42" t="n"/>
       <c r="L26" s="42" t="n"/>
       <c r="M26" s="42" t="n"/>
       <c r="T26" s="4" t="n"/>
@@ -1620,14 +1554,8 @@
       <c r="G27" s="69" t="n"/>
       <c r="H27" s="42" t="n"/>
       <c r="I27" s="42" t="n"/>
-      <c r="J27" s="42" t="inlineStr">
-        <is>
-          <t>2x1</t>
-        </is>
-      </c>
-      <c r="K27" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J27" s="42" t="n"/>
+      <c r="K27" s="42" t="n"/>
       <c r="L27" s="42" t="n"/>
       <c r="M27" s="42" t="n"/>
       <c r="T27" s="4" t="n"/>
@@ -1648,14 +1576,8 @@
       <c r="G28" s="42" t="n"/>
       <c r="H28" s="42" t="n"/>
       <c r="I28" s="34" t="n"/>
-      <c r="J28" s="42" t="inlineStr">
-        <is>
-          <t>1x1</t>
-        </is>
-      </c>
-      <c r="K28" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J28" s="42" t="n"/>
+      <c r="K28" s="42" t="n"/>
       <c r="L28" s="42" t="n"/>
       <c r="M28" s="42" t="n"/>
       <c r="N28" s="42" t="n"/>
@@ -1677,14 +1599,8 @@
       <c r="G29" s="68" t="n"/>
       <c r="H29" s="42" t="n"/>
       <c r="I29" s="42" t="n"/>
-      <c r="J29" s="42" t="inlineStr">
-        <is>
-          <t>2x1</t>
-        </is>
-      </c>
-      <c r="K29" s="42" t="n">
-        <v>5</v>
-      </c>
+      <c r="J29" s="42" t="n"/>
+      <c r="K29" s="42" t="n"/>
       <c r="L29" s="42" t="n"/>
       <c r="M29" s="42" t="n"/>
       <c r="T29" s="5" t="n"/>
@@ -1705,14 +1621,8 @@
       <c r="G30" s="69" t="n"/>
       <c r="H30" s="42" t="n"/>
       <c r="I30" s="42" t="n"/>
-      <c r="J30" s="42" t="inlineStr">
-        <is>
-          <t>3x1</t>
-        </is>
-      </c>
-      <c r="K30" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J30" s="42" t="n"/>
+      <c r="K30" s="42" t="n"/>
       <c r="L30" s="42" t="n"/>
       <c r="M30" s="42" t="n"/>
       <c r="T30" s="5" t="n"/>
@@ -1733,14 +1643,8 @@
       <c r="G31" s="42" t="n"/>
       <c r="H31" s="42" t="n"/>
       <c r="I31" s="42" t="n"/>
-      <c r="J31" s="42" t="inlineStr">
-        <is>
-          <t>3x1</t>
-        </is>
-      </c>
-      <c r="K31" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J31" s="42" t="n"/>
+      <c r="K31" s="42" t="n"/>
       <c r="L31" s="42" t="n"/>
       <c r="M31" s="42" t="n"/>
       <c r="N31" s="42" t="n"/>
@@ -1762,14 +1666,8 @@
       <c r="G32" s="68" t="n"/>
       <c r="H32" s="42" t="n"/>
       <c r="I32" s="42" t="n"/>
-      <c r="J32" s="42" t="inlineStr">
-        <is>
-          <t>2x1</t>
-        </is>
-      </c>
-      <c r="K32" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J32" s="42" t="n"/>
+      <c r="K32" s="42" t="n"/>
       <c r="L32" s="42" t="n"/>
       <c r="M32" s="42" t="n"/>
       <c r="T32" s="5" t="n"/>
@@ -1790,14 +1688,8 @@
       <c r="G33" s="68" t="n"/>
       <c r="H33" s="42" t="n"/>
       <c r="I33" s="42" t="n"/>
-      <c r="J33" s="42" t="inlineStr">
-        <is>
-          <t>3x1</t>
-        </is>
-      </c>
-      <c r="K33" s="42" t="n">
-        <v>10</v>
-      </c>
+      <c r="J33" s="42" t="n"/>
+      <c r="K33" s="42" t="n"/>
       <c r="L33" s="42" t="n"/>
       <c r="M33" s="42" t="n"/>
       <c r="T33" s="5" t="n"/>
@@ -5646,7 +5538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:P70"/>
+  <dimension ref="A2:S70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="9.140625" customWidth="1" style="36" min="1" max="1"/>
@@ -6287,23 +6179,11 @@
       <c r="G10" s="42" t="n"/>
       <c r="H10" s="42" t="n"/>
       <c r="I10" s="42" t="n"/>
-      <c r="J10" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K10" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L10" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J10" s="42" t="n"/>
+      <c r="K10" s="42" t="n"/>
+      <c r="L10" s="42" t="n"/>
       <c r="M10" s="42" t="n"/>
-      <c r="N10" s="42" t="inlineStr">
-        <is>
-          <t>Awuliti</t>
-        </is>
-      </c>
+      <c r="N10" s="42" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="68" t="n"/>
@@ -6315,17 +6195,9 @@
       <c r="G11" s="68" t="n"/>
       <c r="H11" s="42" t="n"/>
       <c r="I11" s="42" t="n"/>
-      <c r="J11" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L11" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J11" s="42" t="n"/>
+      <c r="K11" s="42" t="n"/>
+      <c r="L11" s="42" t="n"/>
       <c r="M11" s="42" t="n"/>
     </row>
     <row r="12">
@@ -6353,17 +6225,9 @@
       <c r="G13" s="69" t="n"/>
       <c r="H13" s="42" t="n"/>
       <c r="I13" s="42" t="n"/>
-      <c r="J13" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L13" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J13" s="42" t="n"/>
+      <c r="K13" s="42" t="n"/>
+      <c r="L13" s="42" t="n"/>
       <c r="M13" s="42" t="n"/>
     </row>
     <row r="14">
@@ -6376,23 +6240,11 @@
       <c r="G14" s="42" t="n"/>
       <c r="H14" s="42" t="n"/>
       <c r="I14" s="42" t="n"/>
-      <c r="J14" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K14" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L14" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J14" s="42" t="n"/>
+      <c r="K14" s="42" t="n"/>
+      <c r="L14" s="42" t="n"/>
       <c r="M14" s="42" t="n"/>
-      <c r="N14" s="42" t="inlineStr">
-        <is>
-          <t>Amberi</t>
-        </is>
-      </c>
+      <c r="N14" s="42" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="68" t="n"/>
@@ -6404,17 +6256,9 @@
       <c r="G15" s="68" t="n"/>
       <c r="H15" s="42" t="n"/>
       <c r="I15" s="42" t="n"/>
-      <c r="J15" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" s="42" t="n">
-        <v>5</v>
-      </c>
-      <c r="L15" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J15" s="42" t="n"/>
+      <c r="K15" s="42" t="n"/>
+      <c r="L15" s="42" t="n"/>
       <c r="M15" s="42" t="n"/>
     </row>
     <row r="16">
@@ -6443,23 +6287,11 @@
       <c r="G18" s="42" t="n"/>
       <c r="H18" s="42" t="n"/>
       <c r="I18" s="42" t="n"/>
-      <c r="J18" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K18" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L18" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J18" s="42" t="n"/>
+      <c r="K18" s="42" t="n"/>
+      <c r="L18" s="42" t="n"/>
       <c r="M18" s="42" t="n"/>
-      <c r="N18" s="42" t="inlineStr">
-        <is>
-          <t>Tanggobu</t>
-        </is>
-      </c>
+      <c r="N18" s="42" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="68" t="n"/>
@@ -6471,17 +6303,9 @@
       <c r="G19" s="68" t="n"/>
       <c r="H19" s="42" t="n"/>
       <c r="I19" s="42" t="n"/>
-      <c r="J19" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K19" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L19" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J19" s="42" t="n"/>
+      <c r="K19" s="42" t="n"/>
+      <c r="L19" s="42" t="n"/>
       <c r="M19" s="42" t="n"/>
     </row>
     <row r="20">
@@ -6494,17 +6318,9 @@
       <c r="G20" s="68" t="n"/>
       <c r="H20" s="42" t="n"/>
       <c r="I20" s="42" t="n"/>
-      <c r="J20" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K20" s="42" t="n">
-        <v>5</v>
-      </c>
-      <c r="L20" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J20" s="42" t="n"/>
+      <c r="K20" s="42" t="n"/>
+      <c r="L20" s="42" t="n"/>
       <c r="M20" s="42" t="n"/>
     </row>
     <row r="21">
@@ -6517,17 +6333,9 @@
       <c r="G21" s="69" t="n"/>
       <c r="H21" s="42" t="n"/>
       <c r="I21" s="42" t="n"/>
-      <c r="J21" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K21" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L21" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J21" s="42" t="n"/>
+      <c r="K21" s="42" t="n"/>
+      <c r="L21" s="42" t="n"/>
       <c r="M21" s="42" t="n"/>
     </row>
     <row r="22"/>
@@ -6542,23 +6350,11 @@
       <c r="G24" s="42" t="n"/>
       <c r="H24" s="42" t="n"/>
       <c r="I24" s="42" t="n"/>
-      <c r="J24" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K24" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L24" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J24" s="42" t="n"/>
+      <c r="K24" s="42" t="n"/>
+      <c r="L24" s="42" t="n"/>
       <c r="M24" s="42" t="n"/>
-      <c r="N24" s="42" t="inlineStr">
-        <is>
-          <t>Awuliti</t>
-        </is>
-      </c>
+      <c r="N24" s="42" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="68" t="n"/>
@@ -6570,17 +6366,9 @@
       <c r="G25" s="68" t="n"/>
       <c r="H25" s="42" t="n"/>
       <c r="I25" s="42" t="n"/>
-      <c r="J25" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K25" s="42" t="n">
-        <v>10</v>
-      </c>
-      <c r="L25" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J25" s="42" t="n"/>
+      <c r="K25" s="42" t="n"/>
+      <c r="L25" s="42" t="n"/>
       <c r="M25" s="42" t="n"/>
     </row>
     <row r="26">
@@ -6611,23 +6399,11 @@
       <c r="G30" s="42" t="n"/>
       <c r="H30" s="42" t="n"/>
       <c r="I30" s="42" t="n"/>
-      <c r="J30" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="L30" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J30" s="42" t="n"/>
+      <c r="K30" s="42" t="n"/>
+      <c r="L30" s="42" t="n"/>
       <c r="M30" s="42" t="n"/>
-      <c r="N30" s="42" t="inlineStr">
-        <is>
-          <t>Amberi</t>
-        </is>
-      </c>
+      <c r="N30" s="42" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="68" t="n"/>
@@ -6639,17 +6415,9 @@
       <c r="G31" s="68" t="n"/>
       <c r="H31" s="42" t="n"/>
       <c r="I31" s="42" t="n"/>
-      <c r="J31" s="42" t="n">
-        <v>0</v>
-      </c>
-      <c r="K31" s="42" t="n">
-        <v>1</v>
-      </c>
-      <c r="L31" s="42" t="inlineStr">
-        <is>
-          <t>Setelah makan</t>
-        </is>
-      </c>
+      <c r="J31" s="42" t="n"/>
+      <c r="K31" s="42" t="n"/>
+      <c r="L31" s="42" t="n"/>
       <c r="M31" s="42" t="n"/>
     </row>
     <row r="32">

</xml_diff>

<commit_message>
fix: bongkar sel gabungan tersisa di template POR yang bikin data nyasar
</commit_message>
<xml_diff>
--- a/public/tpl_por.xlsx
+++ b/public/tpl_por.xlsx
@@ -456,7 +456,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="83">
+  <cellXfs count="81">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -609,8 +609,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="20" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1229,13 +1227,6 @@
       <c r="Z10" s="4" t="n"/>
     </row>
     <row r="11" ht="11.25" customHeight="1" s="36">
-      <c r="A11" s="68" t="n"/>
-      <c r="B11" s="68" t="n"/>
-      <c r="C11" s="68" t="n"/>
-      <c r="D11" s="68" t="n"/>
-      <c r="E11" s="68" t="n"/>
-      <c r="F11" s="68" t="n"/>
-      <c r="G11" s="68" t="n"/>
       <c r="H11" s="42" t="n"/>
       <c r="I11" s="34" t="n"/>
       <c r="J11" s="42" t="n"/>
@@ -1251,13 +1242,6 @@
       <c r="Z11" s="4" t="n"/>
     </row>
     <row r="12" ht="11.25" customHeight="1" s="36">
-      <c r="A12" s="68" t="n"/>
-      <c r="B12" s="68" t="n"/>
-      <c r="C12" s="68" t="n"/>
-      <c r="D12" s="68" t="n"/>
-      <c r="E12" s="68" t="n"/>
-      <c r="F12" s="68" t="n"/>
-      <c r="G12" s="68" t="n"/>
       <c r="H12" s="42" t="n"/>
       <c r="I12" s="34" t="n"/>
       <c r="J12" s="42" t="n"/>
@@ -1273,13 +1257,6 @@
       <c r="Z12" s="4" t="n"/>
     </row>
     <row r="13" ht="11.25" customHeight="1" s="36">
-      <c r="A13" s="69" t="n"/>
-      <c r="B13" s="69" t="n"/>
-      <c r="C13" s="69" t="n"/>
-      <c r="D13" s="69" t="n"/>
-      <c r="E13" s="69" t="n"/>
-      <c r="F13" s="69" t="n"/>
-      <c r="G13" s="69" t="n"/>
       <c r="H13" s="42" t="n"/>
       <c r="I13" s="34" t="n"/>
       <c r="J13" s="42" t="n"/>
@@ -1318,13 +1295,6 @@
       <c r="Z14" s="4" t="n"/>
     </row>
     <row r="15" hidden="1" ht="34.5" customHeight="1" s="36">
-      <c r="A15" s="68" t="n"/>
-      <c r="B15" s="68" t="n"/>
-      <c r="C15" s="68" t="n"/>
-      <c r="D15" s="68" t="n"/>
-      <c r="E15" s="68" t="n"/>
-      <c r="F15" s="68" t="n"/>
-      <c r="G15" s="68" t="n"/>
       <c r="H15" s="42" t="n"/>
       <c r="I15" s="42" t="n"/>
       <c r="J15" s="42" t="n"/>
@@ -1340,13 +1310,6 @@
       <c r="Z15" s="4" t="n"/>
     </row>
     <row r="16" ht="11.25" customHeight="1" s="36">
-      <c r="A16" s="69" t="n"/>
-      <c r="B16" s="69" t="n"/>
-      <c r="C16" s="69" t="n"/>
-      <c r="D16" s="69" t="n"/>
-      <c r="E16" s="69" t="n"/>
-      <c r="F16" s="69" t="n"/>
-      <c r="G16" s="69" t="n"/>
       <c r="H16" s="42" t="n"/>
       <c r="I16" s="42" t="n"/>
       <c r="J16" s="42" t="n"/>
@@ -1394,13 +1357,6 @@
       <c r="Z18" s="4" t="n"/>
     </row>
     <row r="19" ht="11.25" customHeight="1" s="36">
-      <c r="A19" s="68" t="n"/>
-      <c r="B19" s="68" t="n"/>
-      <c r="C19" s="68" t="n"/>
-      <c r="D19" s="68" t="n"/>
-      <c r="E19" s="68" t="n"/>
-      <c r="F19" s="68" t="n"/>
-      <c r="G19" s="68" t="n"/>
       <c r="H19" s="42" t="n"/>
       <c r="I19" s="42" t="n"/>
       <c r="J19" s="42" t="n"/>
@@ -1416,13 +1372,6 @@
       <c r="Z19" s="4" t="n"/>
     </row>
     <row r="20" ht="11.25" customHeight="1" s="36">
-      <c r="A20" s="68" t="n"/>
-      <c r="B20" s="68" t="n"/>
-      <c r="C20" s="68" t="n"/>
-      <c r="D20" s="68" t="n"/>
-      <c r="E20" s="68" t="n"/>
-      <c r="F20" s="68" t="n"/>
-      <c r="G20" s="68" t="n"/>
       <c r="H20" s="42" t="n"/>
       <c r="I20" s="42" t="n"/>
       <c r="J20" s="42" t="n"/>
@@ -1438,13 +1387,6 @@
       <c r="Z20" s="4" t="n"/>
     </row>
     <row r="21" ht="11.25" customHeight="1" s="36">
-      <c r="A21" s="69" t="n"/>
-      <c r="B21" s="69" t="n"/>
-      <c r="C21" s="69" t="n"/>
-      <c r="D21" s="69" t="n"/>
-      <c r="E21" s="69" t="n"/>
-      <c r="F21" s="69" t="n"/>
-      <c r="G21" s="69" t="n"/>
       <c r="H21" s="42" t="n"/>
       <c r="I21" s="42" t="n"/>
       <c r="J21" s="42" t="n"/>
@@ -1501,13 +1443,6 @@
       <c r="Z24" s="4" t="n"/>
     </row>
     <row r="25" ht="11.25" customHeight="1" s="36">
-      <c r="A25" s="68" t="n"/>
-      <c r="B25" s="68" t="n"/>
-      <c r="C25" s="68" t="n"/>
-      <c r="D25" s="68" t="n"/>
-      <c r="E25" s="68" t="n"/>
-      <c r="F25" s="68" t="n"/>
-      <c r="G25" s="68" t="n"/>
       <c r="H25" s="42" t="n"/>
       <c r="I25" s="42" t="n"/>
       <c r="J25" s="42" t="n"/>
@@ -1523,13 +1458,6 @@
       <c r="Z25" s="4" t="n"/>
     </row>
     <row r="26" ht="11.25" customHeight="1" s="36">
-      <c r="A26" s="68" t="n"/>
-      <c r="B26" s="68" t="n"/>
-      <c r="C26" s="68" t="n"/>
-      <c r="D26" s="68" t="n"/>
-      <c r="E26" s="68" t="n"/>
-      <c r="F26" s="68" t="n"/>
-      <c r="G26" s="68" t="n"/>
       <c r="H26" s="42" t="n"/>
       <c r="I26" s="42" t="n"/>
       <c r="J26" s="42" t="n"/>
@@ -1545,13 +1473,6 @@
       <c r="Z26" s="4" t="n"/>
     </row>
     <row r="27" ht="11.25" customHeight="1" s="36">
-      <c r="A27" s="69" t="n"/>
-      <c r="B27" s="69" t="n"/>
-      <c r="C27" s="69" t="n"/>
-      <c r="D27" s="69" t="n"/>
-      <c r="E27" s="69" t="n"/>
-      <c r="F27" s="69" t="n"/>
-      <c r="G27" s="69" t="n"/>
       <c r="H27" s="42" t="n"/>
       <c r="I27" s="42" t="n"/>
       <c r="J27" s="42" t="n"/>
@@ -1590,13 +1511,6 @@
       <c r="Z28" s="4" t="n"/>
     </row>
     <row r="29" ht="13.5" customHeight="1" s="36">
-      <c r="A29" s="68" t="n"/>
-      <c r="B29" s="68" t="n"/>
-      <c r="C29" s="68" t="n"/>
-      <c r="D29" s="68" t="n"/>
-      <c r="E29" s="68" t="n"/>
-      <c r="F29" s="68" t="n"/>
-      <c r="G29" s="68" t="n"/>
       <c r="H29" s="42" t="n"/>
       <c r="I29" s="42" t="n"/>
       <c r="J29" s="42" t="n"/>
@@ -1612,13 +1526,6 @@
       <c r="Z29" s="5" t="n"/>
     </row>
     <row r="30" ht="13.5" customHeight="1" s="36">
-      <c r="A30" s="69" t="n"/>
-      <c r="B30" s="69" t="n"/>
-      <c r="C30" s="69" t="n"/>
-      <c r="D30" s="69" t="n"/>
-      <c r="E30" s="69" t="n"/>
-      <c r="F30" s="69" t="n"/>
-      <c r="G30" s="69" t="n"/>
       <c r="H30" s="42" t="n"/>
       <c r="I30" s="42" t="n"/>
       <c r="J30" s="42" t="n"/>
@@ -1657,13 +1564,6 @@
       <c r="Z31" s="5" t="n"/>
     </row>
     <row r="32" ht="13.5" customHeight="1" s="36">
-      <c r="A32" s="68" t="n"/>
-      <c r="B32" s="68" t="n"/>
-      <c r="C32" s="68" t="n"/>
-      <c r="D32" s="68" t="n"/>
-      <c r="E32" s="68" t="n"/>
-      <c r="F32" s="68" t="n"/>
-      <c r="G32" s="68" t="n"/>
       <c r="H32" s="42" t="n"/>
       <c r="I32" s="42" t="n"/>
       <c r="J32" s="42" t="n"/>
@@ -1679,13 +1579,6 @@
       <c r="Z32" s="5" t="n"/>
     </row>
     <row r="33" ht="13.5" customHeight="1" s="36">
-      <c r="A33" s="68" t="n"/>
-      <c r="B33" s="68" t="n"/>
-      <c r="C33" s="68" t="n"/>
-      <c r="D33" s="68" t="n"/>
-      <c r="E33" s="68" t="n"/>
-      <c r="F33" s="68" t="n"/>
-      <c r="G33" s="68" t="n"/>
       <c r="H33" s="42" t="n"/>
       <c r="I33" s="42" t="n"/>
       <c r="J33" s="42" t="n"/>
@@ -1701,13 +1594,6 @@
       <c r="Z33" s="5" t="n"/>
     </row>
     <row r="34" ht="13.5" customHeight="1" s="36">
-      <c r="A34" s="69" t="n"/>
-      <c r="B34" s="69" t="n"/>
-      <c r="C34" s="69" t="n"/>
-      <c r="D34" s="69" t="n"/>
-      <c r="E34" s="69" t="n"/>
-      <c r="F34" s="69" t="n"/>
-      <c r="G34" s="69" t="n"/>
       <c r="H34" s="42" t="n"/>
       <c r="I34" s="42" t="n"/>
       <c r="J34" s="42" t="n"/>
@@ -5480,52 +5366,10 @@
     <row r="996" ht="13.5" customHeight="1" s="36"/>
     <row r="997" ht="13.5" customHeight="1" s="36"/>
   </sheetData>
-  <mergeCells count="45">
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="B31:B34"/>
-    <mergeCell ref="D31:D34"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="F28:F30"/>
-    <mergeCell ref="G14:G16"/>
-    <mergeCell ref="F24:F27"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="C24:C27"/>
+  <mergeCells count="3">
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="H9:I9"/>
-    <mergeCell ref="C10:C13"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="F14:F16"/>
-    <mergeCell ref="G10:G13"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="G18:G21"/>
-    <mergeCell ref="E31:E34"/>
-    <mergeCell ref="A28:A30"/>
-    <mergeCell ref="C28:C30"/>
-    <mergeCell ref="C31:C34"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="G24:G27"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="F31:F34"/>
-    <mergeCell ref="F10:F13"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="B24:B27"/>
-    <mergeCell ref="D24:D27"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="E24:E27"/>
-    <mergeCell ref="A31:A34"/>
-    <mergeCell ref="G31:G34"/>
-    <mergeCell ref="B14:B16"/>
-    <mergeCell ref="G28:G30"/>
     <mergeCell ref="H8:I8"/>
-    <mergeCell ref="A24:A27"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="D28:D30"/>
-    <mergeCell ref="C18:C21"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -6186,13 +6030,6 @@
       <c r="N10" s="42" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="68" t="n"/>
-      <c r="B11" s="68" t="n"/>
-      <c r="C11" s="68" t="n"/>
-      <c r="D11" s="68" t="n"/>
-      <c r="E11" s="68" t="n"/>
-      <c r="F11" s="68" t="n"/>
-      <c r="G11" s="68" t="n"/>
       <c r="H11" s="42" t="n"/>
       <c r="I11" s="42" t="n"/>
       <c r="J11" s="42" t="n"/>
@@ -6201,13 +6038,6 @@
       <c r="M11" s="42" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="68" t="n"/>
-      <c r="B12" s="68" t="n"/>
-      <c r="C12" s="68" t="n"/>
-      <c r="D12" s="68" t="n"/>
-      <c r="E12" s="68" t="n"/>
-      <c r="F12" s="68" t="n"/>
-      <c r="G12" s="68" t="n"/>
       <c r="H12" s="42" t="n"/>
       <c r="I12" s="42" t="n"/>
       <c r="J12" s="42" t="n"/>
@@ -6216,13 +6046,6 @@
       <c r="M12" s="42" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="69" t="n"/>
-      <c r="B13" s="69" t="n"/>
-      <c r="C13" s="69" t="n"/>
-      <c r="D13" s="69" t="n"/>
-      <c r="E13" s="69" t="n"/>
-      <c r="F13" s="69" t="n"/>
-      <c r="G13" s="69" t="n"/>
       <c r="H13" s="42" t="n"/>
       <c r="I13" s="42" t="n"/>
       <c r="J13" s="42" t="n"/>
@@ -6247,13 +6070,6 @@
       <c r="N14" s="42" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="68" t="n"/>
-      <c r="B15" s="68" t="n"/>
-      <c r="C15" s="68" t="n"/>
-      <c r="D15" s="68" t="n"/>
-      <c r="E15" s="68" t="n"/>
-      <c r="F15" s="68" t="n"/>
-      <c r="G15" s="68" t="n"/>
       <c r="H15" s="42" t="n"/>
       <c r="I15" s="42" t="n"/>
       <c r="J15" s="42" t="n"/>
@@ -6262,13 +6078,6 @@
       <c r="M15" s="42" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="69" t="n"/>
-      <c r="B16" s="69" t="n"/>
-      <c r="C16" s="69" t="n"/>
-      <c r="D16" s="69" t="n"/>
-      <c r="E16" s="69" t="n"/>
-      <c r="F16" s="69" t="n"/>
-      <c r="G16" s="69" t="n"/>
       <c r="H16" s="42" t="n"/>
       <c r="I16" s="42" t="n"/>
       <c r="J16" s="42" t="n"/>
@@ -6294,13 +6103,6 @@
       <c r="N18" s="42" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="68" t="n"/>
-      <c r="B19" s="68" t="n"/>
-      <c r="C19" s="68" t="n"/>
-      <c r="D19" s="68" t="n"/>
-      <c r="E19" s="68" t="n"/>
-      <c r="F19" s="68" t="n"/>
-      <c r="G19" s="68" t="n"/>
       <c r="H19" s="42" t="n"/>
       <c r="I19" s="42" t="n"/>
       <c r="J19" s="42" t="n"/>
@@ -6309,13 +6111,6 @@
       <c r="M19" s="42" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="68" t="n"/>
-      <c r="B20" s="68" t="n"/>
-      <c r="C20" s="68" t="n"/>
-      <c r="D20" s="68" t="n"/>
-      <c r="E20" s="68" t="n"/>
-      <c r="F20" s="68" t="n"/>
-      <c r="G20" s="68" t="n"/>
       <c r="H20" s="42" t="n"/>
       <c r="I20" s="42" t="n"/>
       <c r="J20" s="42" t="n"/>
@@ -6324,13 +6119,6 @@
       <c r="M20" s="42" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="69" t="n"/>
-      <c r="B21" s="69" t="n"/>
-      <c r="C21" s="69" t="n"/>
-      <c r="D21" s="69" t="n"/>
-      <c r="E21" s="69" t="n"/>
-      <c r="F21" s="69" t="n"/>
-      <c r="G21" s="69" t="n"/>
       <c r="H21" s="42" t="n"/>
       <c r="I21" s="42" t="n"/>
       <c r="J21" s="42" t="n"/>
@@ -6357,13 +6145,6 @@
       <c r="N24" s="42" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="68" t="n"/>
-      <c r="B25" s="68" t="n"/>
-      <c r="C25" s="68" t="n"/>
-      <c r="D25" s="68" t="n"/>
-      <c r="E25" s="68" t="n"/>
-      <c r="F25" s="68" t="n"/>
-      <c r="G25" s="68" t="n"/>
       <c r="H25" s="42" t="n"/>
       <c r="I25" s="42" t="n"/>
       <c r="J25" s="42" t="n"/>
@@ -6372,13 +6153,6 @@
       <c r="M25" s="42" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="69" t="n"/>
-      <c r="B26" s="69" t="n"/>
-      <c r="C26" s="69" t="n"/>
-      <c r="D26" s="69" t="n"/>
-      <c r="E26" s="69" t="n"/>
-      <c r="F26" s="69" t="n"/>
-      <c r="G26" s="69" t="n"/>
       <c r="H26" s="42" t="n"/>
       <c r="I26" s="42" t="n"/>
       <c r="J26" s="42" t="n"/>
@@ -6406,13 +6180,6 @@
       <c r="N30" s="42" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="68" t="n"/>
-      <c r="B31" s="68" t="n"/>
-      <c r="C31" s="68" t="n"/>
-      <c r="D31" s="68" t="n"/>
-      <c r="E31" s="68" t="n"/>
-      <c r="F31" s="68" t="n"/>
-      <c r="G31" s="68" t="n"/>
       <c r="H31" s="42" t="n"/>
       <c r="I31" s="42" t="n"/>
       <c r="J31" s="42" t="n"/>
@@ -6421,13 +6188,6 @@
       <c r="M31" s="42" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="69" t="n"/>
-      <c r="B32" s="69" t="n"/>
-      <c r="C32" s="69" t="n"/>
-      <c r="D32" s="69" t="n"/>
-      <c r="E32" s="69" t="n"/>
-      <c r="F32" s="69" t="n"/>
-      <c r="G32" s="69" t="n"/>
       <c r="H32" s="42" t="n"/>
       <c r="I32" s="42" t="n"/>
       <c r="J32" s="42" t="n"/>
@@ -6482,45 +6242,10 @@
     <row r="69" ht="15" customHeight="1" s="36"/>
     <row r="70" ht="15" customHeight="1" s="36"/>
   </sheetData>
-  <mergeCells count="38">
-    <mergeCell ref="E18:E21"/>
-    <mergeCell ref="E30:E32"/>
-    <mergeCell ref="G30:G32"/>
-    <mergeCell ref="B18:B21"/>
-    <mergeCell ref="B30:B32"/>
-    <mergeCell ref="G14:G16"/>
-    <mergeCell ref="B24:B26"/>
-    <mergeCell ref="A14:A16"/>
-    <mergeCell ref="D24:D26"/>
-    <mergeCell ref="C10:C13"/>
+  <mergeCells count="3">
     <mergeCell ref="H9:I9"/>
-    <mergeCell ref="D14:D16"/>
-    <mergeCell ref="E10:E13"/>
-    <mergeCell ref="F14:F16"/>
     <mergeCell ref="A2:L2"/>
-    <mergeCell ref="G10:G13"/>
-    <mergeCell ref="D30:D32"/>
-    <mergeCell ref="F18:F21"/>
-    <mergeCell ref="C18:C21"/>
-    <mergeCell ref="G18:G21"/>
-    <mergeCell ref="A24:A26"/>
-    <mergeCell ref="C24:C26"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="A18:A21"/>
-    <mergeCell ref="A30:A32"/>
-    <mergeCell ref="C30:C32"/>
-    <mergeCell ref="D18:D21"/>
-    <mergeCell ref="E24:E26"/>
-    <mergeCell ref="C14:C16"/>
-    <mergeCell ref="F30:F32"/>
-    <mergeCell ref="E14:E16"/>
-    <mergeCell ref="F24:F26"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="B14:B16"/>
     <mergeCell ref="H8:I8"/>
-    <mergeCell ref="G24:G26"/>
-    <mergeCell ref="D10:D13"/>
-    <mergeCell ref="F10:F13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -6726,17 +6451,17 @@
           <t>% Penggunaan</t>
         </is>
       </c>
-      <c r="D19" s="70" t="inlineStr">
+      <c r="D19" s="68" t="inlineStr">
         <is>
           <t>Rerata Item / Lembar Resep (d)</t>
         </is>
       </c>
-      <c r="E19" s="71" t="n"/>
-      <c r="F19" s="71" t="n"/>
-      <c r="G19" s="72" t="n"/>
+      <c r="E19" s="69" t="n"/>
+      <c r="F19" s="69" t="n"/>
+      <c r="G19" s="70" t="n"/>
     </row>
     <row r="20" ht="15" customHeight="1" s="36">
-      <c r="A20" s="73" t="n"/>
+      <c r="A20" s="71" t="n"/>
       <c r="B20" s="17" t="inlineStr">
         <is>
           <t>Antibiotik pada</t>
@@ -6747,13 +6472,13 @@
           <t>Antibiotik pada</t>
         </is>
       </c>
-      <c r="D20" s="74" t="n"/>
-      <c r="E20" s="75" t="n"/>
-      <c r="F20" s="75" t="n"/>
-      <c r="G20" s="76" t="n"/>
+      <c r="D20" s="72" t="n"/>
+      <c r="E20" s="73" t="n"/>
+      <c r="F20" s="73" t="n"/>
+      <c r="G20" s="74" t="n"/>
     </row>
     <row r="21" ht="15" customHeight="1" s="36">
-      <c r="A21" s="73" t="n"/>
+      <c r="A21" s="71" t="n"/>
       <c r="B21" s="17" t="inlineStr">
         <is>
           <t>ISPA Non</t>
@@ -6764,25 +6489,25 @@
           <t>Diare Non</t>
         </is>
       </c>
-      <c r="D21" s="70" t="inlineStr">
+      <c r="D21" s="68" t="inlineStr">
         <is>
           <t>ISPA</t>
         </is>
       </c>
-      <c r="E21" s="70" t="inlineStr">
+      <c r="E21" s="68" t="inlineStr">
         <is>
           <t>Diare</t>
         </is>
       </c>
-      <c r="F21" s="70" t="inlineStr">
+      <c r="F21" s="68" t="inlineStr">
         <is>
           <t>Rata-rata</t>
         </is>
       </c>
-      <c r="G21" s="72" t="n"/>
+      <c r="G21" s="70" t="n"/>
     </row>
     <row r="22" ht="15" customHeight="1" s="36">
-      <c r="A22" s="73" t="n"/>
+      <c r="A22" s="71" t="n"/>
       <c r="B22" s="17" t="inlineStr">
         <is>
           <t>Pneumonia</t>
@@ -6793,13 +6518,13 @@
           <t>Spesifik</t>
         </is>
       </c>
-      <c r="D22" s="73" t="n"/>
-      <c r="E22" s="73" t="n"/>
-      <c r="F22" s="77" t="n"/>
-      <c r="G22" s="78" t="n"/>
+      <c r="D22" s="71" t="n"/>
+      <c r="E22" s="71" t="n"/>
+      <c r="F22" s="75" t="n"/>
+      <c r="G22" s="76" t="n"/>
     </row>
     <row r="23" ht="15" customHeight="1" s="36">
-      <c r="A23" s="79" t="n"/>
+      <c r="A23" s="77" t="n"/>
       <c r="B23" s="18" t="inlineStr">
         <is>
           <t>(a)</t>
@@ -6810,10 +6535,10 @@
           <t>(b)</t>
         </is>
       </c>
-      <c r="D23" s="79" t="n"/>
-      <c r="E23" s="79" t="n"/>
-      <c r="F23" s="74" t="n"/>
-      <c r="G23" s="76" t="n"/>
+      <c r="D23" s="77" t="n"/>
+      <c r="E23" s="77" t="n"/>
+      <c r="F23" s="72" t="n"/>
+      <c r="G23" s="74" t="n"/>
     </row>
     <row r="24" ht="15" customHeight="1" s="36">
       <c r="A24" s="19" t="n"/>
@@ -6829,10 +6554,10 @@
       <c r="E24" s="20" t="n">
         <v>4</v>
       </c>
-      <c r="F24" s="80" t="n">
+      <c r="F24" s="78" t="n">
         <v>5</v>
       </c>
-      <c r="G24" s="81" t="n"/>
+      <c r="G24" s="79" t="n"/>
     </row>
     <row r="25" ht="15" customHeight="1" s="36">
       <c r="A25" s="21" t="inlineStr">
@@ -6844,8 +6569,8 @@
       <c r="C25" s="21" t="n"/>
       <c r="D25" s="21" t="n"/>
       <c r="E25" s="21" t="n"/>
-      <c r="F25" s="82" t="n"/>
-      <c r="G25" s="81" t="n"/>
+      <c r="F25" s="80" t="n"/>
+      <c r="G25" s="79" t="n"/>
     </row>
     <row r="26" ht="14.25" customHeight="1" s="36">
       <c r="A26" s="15" t="n"/>

</xml_diff>